<commit_message>
feat(PDG-38): onboard EU Most Wanted watchlist mapping and config
</commit_message>
<xml_diff>
--- a/data/rules/preNormalization.xlsx
+++ b/data/rules/preNormalization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BADAED8-F35E-44D0-920B-0754785E1DC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{825364ED-ED95-469F-B43D-A6448BC44C0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2170" yWindow="1850" windowWidth="15680" windowHeight="9430" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="94">
   <si>
     <t>source</t>
   </si>
@@ -276,14 +276,48 @@
   <si>
     <t>IMAGE=Photograph|DOCUMENT=Poster|DETAIL_PAGE=Profile|THUMBNAIL=Thumbnail</t>
   </si>
+  <si>
+    <t>EU-MOST-WANTED</t>
+  </si>
+  <si>
+    <t>list.name</t>
+  </si>
+  <si>
+    <t>detail.published</t>
+  </si>
+  <si>
+    <t>list.is_dangerous</t>
+  </si>
+  <si>
+    <t>^(?P&lt;full_name&gt;(?P&lt;last_name&gt;[^,]+),\s*(?P&lt;first_name&gt;.+))$</t>
+  </si>
+  <si>
+    <t>^on\s+(?P&lt;date_added&gt;.+?),\s*last modified on\s+(?P&lt;date_updated&gt;.+)$</t>
+  </si>
+  <si>
+    <t>1=Yes|0=No</t>
+  </si>
+  <si>
+    <t>detail.reporting_phone[]</t>
+  </si>
+  <si>
+    <t>(?P&lt;phone&gt;\+?\d[\d\s./-]*\d)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -381,9 +415,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -392,23 +429,23 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2210,11 +2247,21 @@
       <c r="AA38" s="3"/>
     </row>
     <row r="39" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A39" s="3"/>
-      <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
-      <c r="D39" s="3"/>
-      <c r="E39" s="3"/>
+      <c r="A39" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>89</v>
+      </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
@@ -2239,11 +2286,21 @@
       <c r="AA39" s="3"/>
     </row>
     <row r="40" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A40" s="3"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
-      <c r="D40" s="3"/>
-      <c r="E40" s="3"/>
+      <c r="A40" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>90</v>
+      </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
       <c r="H40" s="3"/>
@@ -2268,11 +2325,21 @@
       <c r="AA40" s="3"/>
     </row>
     <row r="41" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A41" s="3"/>
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
-      <c r="D41" s="3"/>
-      <c r="E41" s="3"/>
+      <c r="A41" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>91</v>
+      </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
@@ -2297,11 +2364,21 @@
       <c r="AA41" s="3"/>
     </row>
     <row r="42" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A42" s="3"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
-      <c r="D42" s="3"/>
-      <c r="E42" s="3"/>
+      <c r="A42" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>

</xml_diff>

<commit_message>
feat(PDG-40): integrate World Bank debarred + other sanctions watchlists
Onboard the World Bank sanctions lists (all-Entity) with their mapping,
pre-normalization and source-config rows.

- watchlistConfigs: WORLD-BANK-DEBARRED and WORLD-BANK-OTHER-SANCTIONS
  configs; the other-sanctions record splits its date_of_sanction range
  into wb_sanction_from/to for Measures EffectiveDate/EndDate.
- preProcessingEngine: add generic resolve_reference handler (keyed
  footnote lookup) and let split_field_regex read nested dotted paths so
  it can split list.date_of_sanction; add CONSTRUCTION to entity keywords.
- rules: mapping/preNormalization/sourceConfig rows for both lists.
- tests: split_field_regex nested/flat/no-match unit coverage and
  WORLD-BANK-OTHER-SANCTIONS golden + conformance onboarding.
</commit_message>
<xml_diff>
--- a/data/rules/preNormalization.xlsx
+++ b/data/rules/preNormalization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{825364ED-ED95-469F-B43D-A6448BC44C0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA11716-0364-46DC-A36C-1DAB861CE23F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2170" yWindow="1850" windowWidth="15680" windowHeight="9430" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1100" yWindow="1100" windowWidth="15680" windowHeight="9430" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="103">
   <si>
     <t>source</t>
   </si>
@@ -235,9 +235,6 @@
     <t>US-MARSHALS-PROFILED-FUGITIVES</t>
   </si>
   <si>
-    <t>attachments[].type</t>
-  </si>
-  <si>
     <t>detail.height</t>
   </si>
   <si>
@@ -274,9 +271,6 @@
     <t>a.k.a.=AKA|f.k.a.=Former Name</t>
   </si>
   <si>
-    <t>IMAGE=Photograph|DOCUMENT=Poster|DETAIL_PAGE=Profile|THUMBNAIL=Thumbnail</t>
-  </si>
-  <si>
     <t>EU-MOST-WANTED</t>
   </si>
   <si>
@@ -303,14 +297,68 @@
   <si>
     <t>(?P&lt;phone&gt;\+?\d[\d\s./-]*\d)</t>
   </si>
+  <si>
+    <t>WORLD-BANK-DEBARRED</t>
+  </si>
+  <si>
+    <t>SUPP_TYPE_CODE</t>
+  </si>
+  <si>
+    <t>F=Entity|I=Individual|C=Entity|U=</t>
+  </si>
+  <si>
+    <t>SUPP_ELIG_STAT</t>
+  </si>
+  <si>
+    <t>DEBARRED=Active|X-DEBARRED=Inactive</t>
+  </si>
+  <si>
+    <t>WORLD-BANK-OTHER-SANCTIONS</t>
+  </si>
+  <si>
+    <t>list.name_raw</t>
+  </si>
+  <si>
+    <t>^(.*?)(?:\s+\*\d+)?\s*$</t>
+  </si>
+  <si>
+    <t>list.sanction_imposed</t>
+  </si>
+  <si>
+    <t>^(.*[A-Za-z])</t>
+  </si>
+  <si>
+    <t>Letter of reprimand=Letter of Reprimand|Conditional Non-debarment=Conditional Non-Debarment|Conditional Non-debarmen=Conditional Non-Debarment</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -415,34 +463,43 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -769,7 +826,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA994"/>
+  <dimension ref="A1:AA993"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="29.83203125" customWidth="1"/>
@@ -1984,10 +2041,10 @@
         <v>71</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>8</v>
+        <v>46</v>
       </c>
-      <c r="E32" s="13" t="s">
-        <v>84</v>
+      <c r="E32" s="3" t="s">
+        <v>72</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
@@ -2013,20 +2070,20 @@
       <c r="AA32" s="3"/>
     </row>
     <row r="33" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="3" t="s">
-        <v>70</v>
+      <c r="A33" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>46</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
@@ -2053,19 +2110,19 @@
     </row>
     <row r="34" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E34" s="3" t="s">
-        <v>76</v>
+      <c r="E34" t="s">
+        <v>79</v>
       </c>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
@@ -2090,9 +2147,9 @@
       <c r="Z34" s="3"/>
       <c r="AA34" s="3"/>
     </row>
-    <row r="35" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:27" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>24</v>
@@ -2101,10 +2158,10 @@
         <v>77</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
-      <c r="E35" t="s">
-        <v>80</v>
+      <c r="E35" s="3" t="s">
+        <v>78</v>
       </c>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
@@ -2129,21 +2186,21 @@
       <c r="Z35" s="3"/>
       <c r="AA35" s="3"/>
     </row>
-    <row r="36" spans="1:27" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A36" s="12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>8</v>
+        <v>49</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
@@ -2170,19 +2227,19 @@
     </row>
     <row r="37" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>49</v>
+        <v>8</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
@@ -2208,20 +2265,20 @@
       <c r="AA37" s="3"/>
     </row>
     <row r="38" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="12" t="s">
-        <v>74</v>
+      <c r="A38" s="3" t="s">
+        <v>83</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C38" s="3" t="s">
-        <v>82</v>
+      <c r="C38" s="13" t="s">
+        <v>84</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>8</v>
+        <v>49</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
@@ -2248,19 +2305,19 @@
     </row>
     <row r="39" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C39" s="14" t="s">
-        <v>86</v>
+      <c r="C39" s="3" t="s">
+        <v>85</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>49</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
@@ -2287,19 +2344,19 @@
     </row>
     <row r="40" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>49</v>
+        <v>8</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
@@ -2326,16 +2383,16 @@
     </row>
     <row r="41" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>8</v>
+        <v>49</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>91</v>
@@ -2365,19 +2422,19 @@
     </row>
     <row r="42" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="3" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>49</v>
+        <v>8</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
@@ -2403,11 +2460,21 @@
       <c r="AA42" s="3"/>
     </row>
     <row r="43" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A43" s="3"/>
-      <c r="B43" s="3"/>
-      <c r="C43" s="3"/>
-      <c r="D43" s="3"/>
-      <c r="E43" s="3"/>
+      <c r="A43" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="B43" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="C43" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="D43" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>96</v>
+      </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
@@ -2432,11 +2499,21 @@
       <c r="AA43" s="3"/>
     </row>
     <row r="44" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A44" s="3"/>
-      <c r="B44" s="3"/>
-      <c r="C44" s="3"/>
-      <c r="D44" s="3"/>
-      <c r="E44" s="3"/>
+      <c r="A44" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="C44" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="D44" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>99</v>
+      </c>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
       <c r="H44" s="3"/>
@@ -2461,11 +2538,21 @@
       <c r="AA44" s="3"/>
     </row>
     <row r="45" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A45" s="3"/>
-      <c r="B45" s="3"/>
-      <c r="C45" s="3"/>
-      <c r="D45" s="3"/>
-      <c r="E45" s="3"/>
+      <c r="A45" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="B45" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C45" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="D45" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>101</v>
+      </c>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
       <c r="H45" s="3"/>
@@ -2489,12 +2576,22 @@
       <c r="Z45" s="3"/>
       <c r="AA45" s="3"/>
     </row>
-    <row r="46" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A46" s="3"/>
-      <c r="B46" s="3"/>
-      <c r="C46" s="3"/>
-      <c r="D46" s="3"/>
-      <c r="E46" s="3"/>
+    <row r="46" spans="1:27" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A46" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="B46" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C46" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="D46" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>102</v>
+      </c>
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
       <c r="H46" s="3"/>
@@ -29981,35 +30078,6 @@
       <c r="Z993" s="3"/>
       <c r="AA993" s="3"/>
     </row>
-    <row r="994" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A994" s="3"/>
-      <c r="B994" s="3"/>
-      <c r="C994" s="3"/>
-      <c r="D994" s="3"/>
-      <c r="E994" s="3"/>
-      <c r="F994" s="3"/>
-      <c r="G994" s="3"/>
-      <c r="H994" s="3"/>
-      <c r="I994" s="3"/>
-      <c r="J994" s="3"/>
-      <c r="K994" s="3"/>
-      <c r="L994" s="3"/>
-      <c r="M994" s="3"/>
-      <c r="N994" s="3"/>
-      <c r="O994" s="3"/>
-      <c r="P994" s="3"/>
-      <c r="Q994" s="3"/>
-      <c r="R994" s="3"/>
-      <c r="S994" s="3"/>
-      <c r="T994" s="3"/>
-      <c r="U994" s="3"/>
-      <c r="V994" s="3"/>
-      <c r="W994" s="3"/>
-      <c r="X994" s="3"/>
-      <c r="Y994" s="3"/>
-      <c r="Z994" s="3"/>
-      <c r="AA994" s="3"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat(PDG-18): strip "Direct:" prefix from PH house member phone in pre-normalization
</commit_message>
<xml_diff>
--- a/data/rules/preNormalization.xlsx
+++ b/data/rules/preNormalization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA11716-0364-46DC-A36C-1DAB861CE23F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE5B916-CD2D-4774-8391-AF055665FF2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="1100" windowWidth="15680" windowHeight="9430" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="106">
   <si>
     <t>source</t>
   </si>
@@ -330,14 +330,30 @@
   <si>
     <t>Letter of reprimand=Letter of Reprimand|Conditional Non-debarment=Conditional Non-Debarment|Conditional Non-debarmen=Conditional Non-Debarment</t>
   </si>
+  <si>
+    <t>PH-HOUSE-MEMBERS</t>
+  </si>
+  <si>
+    <t>detail.direct_phone</t>
+  </si>
+  <si>
+    <t>(\d[\d\s./-]*\d)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -463,9 +479,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -474,23 +493,23 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2616,11 +2635,21 @@
       <c r="AA46" s="3"/>
     </row>
     <row r="47" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3"/>
-      <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
+      <c r="A47" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="B47" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="C47" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="D47" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>105</v>
+      </c>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
       <c r="H47" s="3"/>

</xml_diff>

<commit_message>
feat(PDG-35): integrate ADB debarment and suspension watchlist
</commit_message>
<xml_diff>
--- a/data/rules/preNormalization.xlsx
+++ b/data/rules/preNormalization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE5B916-CD2D-4774-8391-AF055665FF2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C93CB20-1B9B-4777-9594-7BF4981E2885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="1100" windowWidth="15680" windowHeight="9430" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1440" yWindow="1440" windowWidth="15680" windowHeight="9430" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="109">
   <si>
     <t>source</t>
   </si>
@@ -338,6 +338,15 @@
   </si>
   <si>
     <t>(\d[\d\s./-]*\d)</t>
+  </si>
+  <si>
+    <t>attributes.entityType</t>
+  </si>
+  <si>
+    <t>Firm=Entity|Individual=Individual</t>
+  </si>
+  <si>
+    <t>ADB-DEBARMENT-SUSPENSION</t>
   </si>
 </sst>
 </file>
@@ -2674,11 +2683,21 @@
       <c r="AA47" s="3"/>
     </row>
     <row r="48" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A48" s="3"/>
-      <c r="B48" s="3"/>
-      <c r="C48" s="3"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="3"/>
+      <c r="A48" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>107</v>
+      </c>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
       <c r="H48" s="3"/>

</xml_diff>

<commit_message>
checkpoint(PDG-59): WIP before merging staging (date/Duration + adverse-media + scripts reorg)
</commit_message>
<xml_diff>
--- a/data/rules/preNormalization.xlsx
+++ b/data/rules/preNormalization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE5B916-CD2D-4774-8391-AF055665FF2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83765F00-06C6-47B2-93F7-D2AB57DFC722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="1100" windowWidth="15680" windowHeight="9430" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1440" yWindow="1440" windowWidth="15680" windowHeight="9430" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="109">
   <si>
     <t>source</t>
   </si>
@@ -338,6 +338,15 @@
   </si>
   <si>
     <t>(\d[\d\s./-]*\d)</t>
+  </si>
+  <si>
+    <t>ADB-DEBARMENT-SUSPENSION</t>
+  </si>
+  <si>
+    <t>attributes.entityType</t>
+  </si>
+  <si>
+    <t>Firm=Entity|Individual=Individual</t>
   </si>
 </sst>
 </file>
@@ -2674,11 +2683,21 @@
       <c r="AA47" s="3"/>
     </row>
     <row r="48" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A48" s="3"/>
-      <c r="B48" s="3"/>
-      <c r="C48" s="3"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="3"/>
+      <c r="A48" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>108</v>
+      </c>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
       <c r="H48" s="3"/>

</xml_diff>

<commit_message>
feat(PDG-97):Add IDB sanctioned entities watchlist and normalize countries
</commit_message>
<xml_diff>
--- a/data/rules/preNormalization.xlsx
+++ b/data/rules/preNormalization.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FAD5BBB-279D-4264-A830-A3EFB05C98D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76FF4746-4E58-4714-BA85-8E8214F45D89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3340" yWindow="1610" windowWidth="13550" windowHeight="9670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="156">
   <si>
     <t>source</t>
   </si>
@@ -441,14 +441,69 @@
   <si>
     <t>(?is)(?P&lt;type&gt;(?:also|formerly|previously|now)\s+known\s+as|(?:may\s+)?(?:also\s+)?(?:be\s+)?doing\s+business\s+(?:as|under)|(?:also\s+)?d\.?b\.?a\.?(?!\w)|formerly(?:\s+operating\s+as)?|\baka\b|\bf/k/a|\bor\b)\s*:?\s*(?:\(dba\)\s*)?(?P&lt;value&gt;(?:[^()]|\([^()]*\))+?)(?=\s*;|\s*,?\s*\(?\s*(?:(?:also|formerly|previously|now)\s+known\s+as|(?:may\s+)?(?:also\s+)?(?:be\s+)?doing\s+business\s+(?:as|under)|(?:also\s+)?d\.?b\.?a\.?(?!\w)|formerly(?:\s+operating\s+as)?|\baka\b|\bf/k/a|\bor\b)(?!\w)|\s*\)*\s*$)</t>
   </si>
+  <si>
+    <t>IDB_SANCTIONED_ENTITIES</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>(?s)^\s*(.*?)\s*$</t>
+  </si>
+  <si>
+    <t>Nationality</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>From</t>
+  </si>
+  <si>
+    <t>^(\d{4}-\d{2}-\d{2})</t>
+  </si>
+  <si>
+    <t>To</t>
+  </si>
+  <si>
+    <t>^(\d{4}-\d{2}-\d{2}|Ongoing)</t>
+  </si>
+  <si>
+    <t>Tipo de sancion del BID</t>
+  </si>
+  <si>
+    <t>Debarment=Debarment|Debarment w/ conditional release=Debarment|Letter of reprimand=Reprimand|=Debarment</t>
+  </si>
+  <si>
+    <t>idb_measure_type</t>
+  </si>
+  <si>
+    <t>^(Ongoing)$</t>
+  </si>
+  <si>
+    <t>idb_duration</t>
+  </si>
+  <si>
+    <t>target_field</t>
+  </si>
+  <si>
+    <t>China, Hong Kong Special Administrative Region=Hong Kong</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -505,8 +560,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -529,6 +589,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDF3F7"/>
       </patternFill>
     </fill>
   </fills>
@@ -559,100 +624,109 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -994,7 +1068,9 @@
       <c r="E1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2"/>
+      <c r="F1" s="36" t="s">
+        <v>154</v>
+      </c>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
@@ -3655,244 +3731,170 @@
       <c r="Z69" s="2"/>
       <c r="AA69" s="2"/>
     </row>
-    <row r="70" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A70" s="6"/>
-      <c r="B70" s="30"/>
-      <c r="C70" s="6"/>
-      <c r="D70" s="6"/>
-      <c r="E70" s="18"/>
-      <c r="F70" s="2"/>
-      <c r="G70" s="2"/>
-      <c r="H70" s="2"/>
-      <c r="I70" s="2"/>
-      <c r="J70" s="2"/>
-      <c r="K70" s="2"/>
-      <c r="L70" s="2"/>
-      <c r="M70" s="2"/>
-      <c r="N70" s="2"/>
-      <c r="O70" s="2"/>
-      <c r="P70" s="2"/>
-      <c r="Q70" s="2"/>
-      <c r="R70" s="2"/>
-      <c r="S70" s="2"/>
-      <c r="T70" s="2"/>
-      <c r="U70" s="2"/>
-      <c r="V70" s="2"/>
-      <c r="W70" s="2"/>
-      <c r="X70" s="2"/>
-      <c r="Y70" s="2"/>
-      <c r="Z70" s="2"/>
-      <c r="AA70" s="2"/>
-    </row>
-    <row r="71" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A71" s="6"/>
-      <c r="B71" s="30"/>
-      <c r="C71" s="6"/>
-      <c r="D71" s="6"/>
-      <c r="E71" s="18"/>
-      <c r="F71" s="2"/>
-      <c r="G71" s="2"/>
-      <c r="H71" s="2"/>
-      <c r="I71" s="2"/>
-      <c r="J71" s="2"/>
-      <c r="K71" s="2"/>
-      <c r="L71" s="2"/>
-      <c r="M71" s="2"/>
-      <c r="N71" s="2"/>
-      <c r="O71" s="2"/>
-      <c r="P71" s="2"/>
-      <c r="Q71" s="2"/>
-      <c r="R71" s="2"/>
-      <c r="S71" s="2"/>
-      <c r="T71" s="2"/>
-      <c r="U71" s="2"/>
-      <c r="V71" s="2"/>
-      <c r="W71" s="2"/>
-      <c r="X71" s="2"/>
-      <c r="Y71" s="2"/>
-      <c r="Z71" s="2"/>
-      <c r="AA71" s="2"/>
-    </row>
-    <row r="72" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A72" s="6"/>
-      <c r="B72" s="30"/>
-      <c r="C72" s="6"/>
-      <c r="D72" s="6"/>
-      <c r="E72" s="18"/>
-      <c r="F72" s="2"/>
-      <c r="G72" s="2"/>
-      <c r="H72" s="2"/>
-      <c r="I72" s="2"/>
-      <c r="J72" s="2"/>
-      <c r="K72" s="2"/>
-      <c r="L72" s="2"/>
-      <c r="M72" s="2"/>
-      <c r="N72" s="2"/>
-      <c r="O72" s="2"/>
-      <c r="P72" s="2"/>
-      <c r="Q72" s="2"/>
-      <c r="R72" s="2"/>
-      <c r="S72" s="2"/>
-      <c r="T72" s="2"/>
-      <c r="U72" s="2"/>
-      <c r="V72" s="2"/>
-      <c r="W72" s="2"/>
-      <c r="X72" s="2"/>
-      <c r="Y72" s="2"/>
-      <c r="Z72" s="2"/>
-      <c r="AA72" s="2"/>
-    </row>
-    <row r="73" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A73" s="6"/>
-      <c r="B73" s="30"/>
-      <c r="C73" s="6"/>
-      <c r="D73" s="6"/>
-      <c r="E73" s="18"/>
-      <c r="F73" s="2"/>
-      <c r="G73" s="2"/>
-      <c r="H73" s="2"/>
-      <c r="I73" s="2"/>
-      <c r="J73" s="2"/>
-      <c r="K73" s="2"/>
-      <c r="L73" s="2"/>
-      <c r="M73" s="2"/>
-      <c r="N73" s="2"/>
-      <c r="O73" s="2"/>
-      <c r="P73" s="2"/>
-      <c r="Q73" s="2"/>
-      <c r="R73" s="2"/>
-      <c r="S73" s="2"/>
-      <c r="T73" s="2"/>
-      <c r="U73" s="2"/>
-      <c r="V73" s="2"/>
-      <c r="W73" s="2"/>
-      <c r="X73" s="2"/>
-      <c r="Y73" s="2"/>
-      <c r="Z73" s="2"/>
-      <c r="AA73" s="2"/>
-    </row>
-    <row r="74" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A74" s="6"/>
-      <c r="B74" s="30"/>
-      <c r="C74" s="6"/>
-      <c r="D74" s="6"/>
-      <c r="E74" s="18"/>
-      <c r="F74" s="2"/>
-      <c r="G74" s="2"/>
-      <c r="H74" s="2"/>
-      <c r="I74" s="2"/>
-      <c r="J74" s="2"/>
-      <c r="K74" s="2"/>
-      <c r="L74" s="2"/>
-      <c r="M74" s="2"/>
-      <c r="N74" s="2"/>
-      <c r="O74" s="2"/>
-      <c r="P74" s="2"/>
-      <c r="Q74" s="2"/>
-      <c r="R74" s="2"/>
-      <c r="S74" s="2"/>
-      <c r="T74" s="2"/>
-      <c r="U74" s="2"/>
-      <c r="V74" s="2"/>
-      <c r="W74" s="2"/>
-      <c r="X74" s="2"/>
-      <c r="Y74" s="2"/>
-      <c r="Z74" s="2"/>
-      <c r="AA74" s="2"/>
-    </row>
-    <row r="75" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A75" s="6"/>
-      <c r="B75" s="30"/>
-      <c r="C75" s="6"/>
-      <c r="D75" s="6"/>
-      <c r="E75" s="18"/>
-      <c r="F75" s="2"/>
-      <c r="G75" s="2"/>
-      <c r="H75" s="2"/>
-      <c r="I75" s="2"/>
-      <c r="J75" s="2"/>
-      <c r="K75" s="2"/>
-      <c r="L75" s="2"/>
-      <c r="M75" s="2"/>
-      <c r="N75" s="2"/>
-      <c r="O75" s="2"/>
-      <c r="P75" s="2"/>
-      <c r="Q75" s="2"/>
-      <c r="R75" s="2"/>
-      <c r="S75" s="2"/>
-      <c r="T75" s="2"/>
-      <c r="U75" s="2"/>
-      <c r="V75" s="2"/>
-      <c r="W75" s="2"/>
-      <c r="X75" s="2"/>
-      <c r="Y75" s="2"/>
-      <c r="Z75" s="2"/>
-      <c r="AA75" s="2"/>
-    </row>
-    <row r="76" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A76" s="6"/>
-      <c r="B76" s="30"/>
-      <c r="C76" s="6"/>
-      <c r="D76" s="6"/>
-      <c r="E76" s="18"/>
-      <c r="F76" s="2"/>
-      <c r="G76" s="2"/>
-      <c r="H76" s="2"/>
-      <c r="I76" s="2"/>
-      <c r="J76" s="2"/>
-      <c r="K76" s="2"/>
-      <c r="L76" s="2"/>
-      <c r="M76" s="2"/>
-      <c r="N76" s="2"/>
-      <c r="O76" s="2"/>
-      <c r="P76" s="2"/>
-      <c r="Q76" s="2"/>
-      <c r="R76" s="2"/>
-      <c r="S76" s="2"/>
-      <c r="T76" s="2"/>
-      <c r="U76" s="2"/>
-      <c r="V76" s="2"/>
-      <c r="W76" s="2"/>
-      <c r="X76" s="2"/>
-      <c r="Y76" s="2"/>
-      <c r="Z76" s="2"/>
-      <c r="AA76" s="2"/>
-    </row>
-    <row r="77" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A77" s="6"/>
-      <c r="B77" s="30"/>
-      <c r="C77" s="6"/>
-      <c r="D77" s="6"/>
-      <c r="E77" s="18"/>
-      <c r="F77" s="2"/>
-      <c r="G77" s="2"/>
-      <c r="H77" s="2"/>
-      <c r="I77" s="2"/>
-      <c r="J77" s="2"/>
-      <c r="K77" s="2"/>
-      <c r="L77" s="2"/>
-      <c r="M77" s="2"/>
-      <c r="N77" s="2"/>
-      <c r="O77" s="2"/>
-      <c r="P77" s="2"/>
-      <c r="Q77" s="2"/>
-      <c r="R77" s="2"/>
-      <c r="S77" s="2"/>
-      <c r="T77" s="2"/>
-      <c r="U77" s="2"/>
-      <c r="V77" s="2"/>
-      <c r="W77" s="2"/>
-      <c r="X77" s="2"/>
-      <c r="Y77" s="2"/>
-      <c r="Z77" s="2"/>
-      <c r="AA77" s="2"/>
+    <row r="70" spans="1:27" ht="52" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A70" s="34" t="s">
+        <v>140</v>
+      </c>
+      <c r="B70" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C70" s="34" t="s">
+        <v>10</v>
+      </c>
+      <c r="D70" s="34" t="s">
+        <v>8</v>
+      </c>
+      <c r="E70" s="34" t="s">
+        <v>106</v>
+      </c>
+      <c r="F70" s="34"/>
+    </row>
+    <row r="71" spans="1:27" ht="52" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A71" s="35" t="s">
+        <v>140</v>
+      </c>
+      <c r="B71" s="35" t="s">
+        <v>23</v>
+      </c>
+      <c r="C71" s="35" t="s">
+        <v>141</v>
+      </c>
+      <c r="D71" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="E71" s="35" t="s">
+        <v>142</v>
+      </c>
+      <c r="F71" s="35"/>
+    </row>
+    <row r="72" spans="1:27" ht="52" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A72" s="34" t="s">
+        <v>140</v>
+      </c>
+      <c r="B72" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C72" s="34" t="s">
+        <v>143</v>
+      </c>
+      <c r="D72" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="E72" s="34" t="s">
+        <v>142</v>
+      </c>
+      <c r="F72" s="34"/>
+    </row>
+    <row r="73" spans="1:27" ht="52" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A73" s="35" t="s">
+        <v>140</v>
+      </c>
+      <c r="B73" s="35" t="s">
+        <v>23</v>
+      </c>
+      <c r="C73" s="35" t="s">
+        <v>144</v>
+      </c>
+      <c r="D73" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="E73" s="35" t="s">
+        <v>142</v>
+      </c>
+      <c r="F73" s="35"/>
+    </row>
+    <row r="74" spans="1:27" ht="52" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A74" s="34" t="s">
+        <v>140</v>
+      </c>
+      <c r="B74" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C74" s="34" t="s">
+        <v>145</v>
+      </c>
+      <c r="D74" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="E74" s="34" t="s">
+        <v>146</v>
+      </c>
+      <c r="F74" s="34"/>
+    </row>
+    <row r="75" spans="1:27" ht="52" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A75" s="35" t="s">
+        <v>140</v>
+      </c>
+      <c r="B75" s="35" t="s">
+        <v>23</v>
+      </c>
+      <c r="C75" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="D75" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="E75" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="F75" s="35"/>
+    </row>
+    <row r="76" spans="1:27" ht="52" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A76" s="34" t="s">
+        <v>140</v>
+      </c>
+      <c r="B76" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C76" s="34" t="s">
+        <v>149</v>
+      </c>
+      <c r="D76" s="34" t="s">
+        <v>8</v>
+      </c>
+      <c r="E76" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="F76" s="34" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="77" spans="1:27" ht="52" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A77" s="35" t="s">
+        <v>140</v>
+      </c>
+      <c r="B77" s="35" t="s">
+        <v>23</v>
+      </c>
+      <c r="C77" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="D77" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="E77" s="35" t="s">
+        <v>152</v>
+      </c>
+      <c r="F77" s="35" t="s">
+        <v>153</v>
+      </c>
     </row>
     <row r="78" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A78" s="6"/>
-      <c r="B78" s="30"/>
-      <c r="C78" s="6"/>
-      <c r="D78" s="6"/>
-      <c r="E78" s="18"/>
+      <c r="A78" t="s">
+        <v>140</v>
+      </c>
+      <c r="B78" s="35" t="s">
+        <v>23</v>
+      </c>
+      <c r="C78" t="s">
+        <v>143</v>
+      </c>
+      <c r="D78" s="34" t="s">
+        <v>8</v>
+      </c>
+      <c r="E78" t="s">
+        <v>155</v>
+      </c>
       <c r="F78" s="2"/>
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
@@ -3917,11 +3919,21 @@
       <c r="AA78" s="2"/>
     </row>
     <row r="79" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A79" s="6"/>
-      <c r="B79" s="30"/>
-      <c r="C79" s="6"/>
-      <c r="D79" s="6"/>
-      <c r="E79" s="18"/>
+      <c r="A79" t="s">
+        <v>140</v>
+      </c>
+      <c r="B79" s="35" t="s">
+        <v>23</v>
+      </c>
+      <c r="C79" t="s">
+        <v>144</v>
+      </c>
+      <c r="D79" s="34" t="s">
+        <v>8</v>
+      </c>
+      <c r="E79" t="s">
+        <v>155</v>
+      </c>
       <c r="F79" s="2"/>
       <c r="G79" s="2"/>
       <c r="H79" s="2"/>

</xml_diff>

<commit_message>
feat(PDG-102): integrate Interpol UNSC special notices
</commit_message>
<xml_diff>
--- a/data/rules/preNormalization.xlsx
+++ b/data/rules/preNormalization.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76FF4746-4E58-4714-BA85-8E8214F45D89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE0A598-4ABD-42ED-8C4C-A884B45471FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3340" yWindow="1610" windowWidth="13550" windowHeight="9670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="163">
   <si>
     <t>source</t>
   </si>
@@ -488,6 +488,27 @@
   </si>
   <si>
     <t>China, Hong Kong Special Administrative Region=Hong Kong</t>
+  </si>
+  <si>
+    <t>INTERPOL_UNSC_SPECIAL_NOTICES</t>
+  </si>
+  <si>
+    <t>list.record_type</t>
+  </si>
+  <si>
+    <t>Individual=Individual|Entity=Entity</t>
+  </si>
+  <si>
+    <t>detail.identity_documents[].type</t>
+  </si>
+  <si>
+    <t>PASSPORT=Passport|NATIONAL IDENTIFICATION NR=National ID|IDENTITY CARD=Identity Card|OTHER=Other|DRIVING LICENCE=Driving Licence|SOCIAL SECURITY NR=Social Security Number|RESIDENCE PERMIT=Residence Permit|ALIEN REGISTRATION NUMBER=Alien Registration Number</t>
+  </si>
+  <si>
+    <t>detail.purposes[]</t>
+  </si>
+  <si>
+    <t>FOA=Asset Freeze|ARE=Arms Embargo|TRB=Travel Ban</t>
   </si>
 </sst>
 </file>
@@ -3958,11 +3979,21 @@
       <c r="AA79" s="2"/>
     </row>
     <row r="80" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A80" s="6"/>
-      <c r="B80" s="30"/>
-      <c r="C80" s="6"/>
-      <c r="D80" s="6"/>
-      <c r="E80" s="18"/>
+      <c r="A80" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="B80" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E80" s="18" t="s">
+        <v>158</v>
+      </c>
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
       <c r="H80" s="2"/>
@@ -3987,11 +4018,21 @@
       <c r="AA80" s="2"/>
     </row>
     <row r="81" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A81" s="6"/>
-      <c r="B81" s="30"/>
-      <c r="C81" s="6"/>
-      <c r="D81" s="6"/>
-      <c r="E81" s="18"/>
+      <c r="A81" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="B81" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E81" s="18" t="s">
+        <v>62</v>
+      </c>
       <c r="F81" s="2"/>
       <c r="G81" s="2"/>
       <c r="H81" s="2"/>
@@ -4016,11 +4057,21 @@
       <c r="AA81" s="2"/>
     </row>
     <row r="82" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A82" s="6"/>
-      <c r="B82" s="30"/>
-      <c r="C82" s="6"/>
-      <c r="D82" s="6"/>
-      <c r="E82" s="18"/>
+      <c r="A82" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="B82" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D82" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E82" s="18" t="s">
+        <v>160</v>
+      </c>
       <c r="F82" s="2"/>
       <c r="G82" s="2"/>
       <c r="H82" s="2"/>
@@ -4045,11 +4096,21 @@
       <c r="AA82" s="2"/>
     </row>
     <row r="83" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A83" s="6"/>
-      <c r="B83" s="30"/>
-      <c r="C83" s="6"/>
-      <c r="D83" s="6"/>
-      <c r="E83" s="18"/>
+      <c r="A83" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="B83" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="D83" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E83" s="18" t="s">
+        <v>162</v>
+      </c>
       <c r="F83" s="2"/>
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
@@ -4074,10 +4135,18 @@
       <c r="AA83" s="2"/>
     </row>
     <row r="84" spans="1:27" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A84" s="6"/>
-      <c r="B84" s="30"/>
-      <c r="C84" s="6"/>
-      <c r="D84" s="6"/>
+      <c r="A84" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="B84" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D84" s="6" t="s">
+        <v>68</v>
+      </c>
       <c r="E84" s="18"/>
       <c r="F84" s="2"/>
       <c r="G84" s="2"/>

</xml_diff>

<commit_message>
Add Crimestoppers UK Most Wanted watchlist
</commit_message>
<xml_diff>
--- a/data/rules/preNormalization.xlsx
+++ b/data/rules/preNormalization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1387F7AD-95CF-4F95-8CAD-55E85DC2F6C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28E36E48-1D7F-4BC8-9113-35212766A024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1140" yWindow="1140" windowWidth="13550" windowHeight="9670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="205">
   <si>
     <t>source</t>
   </si>
@@ -588,6 +588,54 @@
   <si>
     <t>(?is)^\s*(?!\(?\s*(?:Address\s*:\s*)?(?:None|N/?A|Unknown|Not\s+(?:Available|Provided|Known|Listed)|No\s+(?:Address|Contact(?:\s+Details)?)(?:\s+(?:Identified|Located|Listed|Provided|Available|Known|Given))?)\s*[.!]?\s*\)?\s*$)(.*?)\s*$</t>
   </si>
+  <si>
+    <t>CRIMESTOPPERS_UK_MOST_WANTED</t>
+  </si>
+  <si>
+    <t>detail.page_title</t>
+  </si>
+  <si>
+    <t>(?i)^\s*(.+?)\s+[-–—]\s+Wanted(?:\s+for\b.*)?\s*$</t>
+  </si>
+  <si>
+    <t>cs_name_before_wanted</t>
+  </si>
+  <si>
+    <t>(?i)^\s*Wanted by\s+.+?\s+Police\s*[-–—]\s*(.+?)\s*$</t>
+  </si>
+  <si>
+    <t>cs_name_after_police</t>
+  </si>
+  <si>
+    <t>$</t>
+  </si>
+  <si>
+    <t>first_non_empty</t>
+  </si>
+  <si>
+    <t>detail.suspect_name|cs_name_before_wanted|cs_name_after_police</t>
+  </si>
+  <si>
+    <t>cs_primary_name</t>
+  </si>
+  <si>
+    <t>detail.nickname</t>
+  </si>
+  <si>
+    <t>\s*((?:(?i:N/A)|[^,;/\r\n])+?)\s*(?:\s*[,;/]\s*|\s+(?i:and)\s+|(?&lt;=[A-Z])\.\s+(?=[A-Z])|$)</t>
+  </si>
+  <si>
+    <t>cs_aliases</t>
+  </si>
+  <si>
+    <t>detail.facial_hair</t>
+  </si>
+  <si>
+    <t>None=None (as reported)</t>
+  </si>
+  <si>
+    <t>cs_facial_hair</t>
+  </si>
 </sst>
 </file>
 
@@ -1027,7 +1075,7 @@
   <dimension ref="A1:AA994"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
-    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="1" max="1" width="46.25" customWidth="1"/>
     <col min="2" max="2" width="10.6640625" style="9"/>
     <col min="3" max="3" width="45.33203125" customWidth="1"/>
     <col min="4" max="4" width="29.33203125" customWidth="1"/>
@@ -4792,12 +4840,24 @@
       <c r="AA96" s="1"/>
     </row>
     <row r="97" spans="1:27" ht="16" customHeight="1" thickBot="1">
-      <c r="A97" s="3"/>
-      <c r="B97" s="8"/>
-      <c r="C97" s="3"/>
-      <c r="D97" s="4"/>
-      <c r="E97" s="5"/>
-      <c r="F97" s="1"/>
+      <c r="A97" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B97" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E97" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="F97" s="1" t="s">
+        <v>192</v>
+      </c>
       <c r="G97" s="1"/>
       <c r="H97" s="1"/>
       <c r="I97" s="1"/>
@@ -4821,12 +4881,24 @@
       <c r="AA97" s="1"/>
     </row>
     <row r="98" spans="1:27" ht="16" customHeight="1" thickBot="1">
-      <c r="A98" s="3"/>
-      <c r="B98" s="8"/>
-      <c r="C98" s="3"/>
-      <c r="D98" s="4"/>
-      <c r="E98" s="5"/>
-      <c r="F98" s="1"/>
+      <c r="A98" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B98" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C98" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E98" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="F98" s="1" t="s">
+        <v>194</v>
+      </c>
       <c r="G98" s="1"/>
       <c r="H98" s="1"/>
       <c r="I98" s="1"/>
@@ -4850,12 +4922,24 @@
       <c r="AA98" s="1"/>
     </row>
     <row r="99" spans="1:27" ht="16" customHeight="1" thickBot="1">
-      <c r="A99" s="3"/>
-      <c r="B99" s="8"/>
-      <c r="C99" s="3"/>
-      <c r="D99" s="3"/>
-      <c r="E99" s="5"/>
-      <c r="F99" s="1"/>
+      <c r="A99" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B99" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C99" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="D99" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="E99" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="F99" s="1" t="s">
+        <v>198</v>
+      </c>
       <c r="G99" s="1"/>
       <c r="H99" s="1"/>
       <c r="I99" s="1"/>
@@ -4879,12 +4963,24 @@
       <c r="AA99" s="1"/>
     </row>
     <row r="100" spans="1:27" ht="16" customHeight="1" thickBot="1">
-      <c r="A100" s="3"/>
-      <c r="B100" s="8"/>
-      <c r="C100" s="3"/>
-      <c r="D100" s="3"/>
-      <c r="E100" s="5"/>
-      <c r="F100" s="1"/>
+      <c r="A100" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B100" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C100" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="D100" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="E100" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="F100" s="1" t="s">
+        <v>201</v>
+      </c>
       <c r="G100" s="1"/>
       <c r="H100" s="1"/>
       <c r="I100" s="1"/>
@@ -4908,12 +5004,24 @@
       <c r="AA100" s="1"/>
     </row>
     <row r="101" spans="1:27" ht="16" customHeight="1" thickBot="1">
-      <c r="A101" s="3"/>
-      <c r="B101" s="8"/>
-      <c r="C101" s="3"/>
-      <c r="D101" s="3"/>
-      <c r="E101" s="5"/>
-      <c r="F101" s="1"/>
+      <c r="A101" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B101" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C101" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="D101" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E101" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F101" s="1" t="s">
+        <v>204</v>
+      </c>
       <c r="G101" s="1"/>
       <c r="H101" s="1"/>
       <c r="I101" s="1"/>

</xml_diff>